<commit_message>
Update widget model_id in Analisa.ipynb and refresh Dataset Analisis Trading.xlsx
</commit_message>
<xml_diff>
--- a/Dataset Analisis Trading.xlsx
+++ b/Dataset Analisis Trading.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\Trading Analysis\FibPath Analyzer V2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\Fibpath Analyzer\fibpath-analyzer-v3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45BB7239-6757-4ECC-8B7A-AE385450F858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19FCDB43-0DE2-40BA-8ED9-863C880915C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="13403" windowWidth="21795" windowHeight="12975" xr2:uid="{0FBFC3C1-39E9-48C7-94FA-7929923CC50D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1339" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1355" uniqueCount="168">
   <si>
     <t>Trend</t>
   </si>
@@ -532,6 +532,12 @@
   </si>
   <si>
     <t>17,8</t>
+  </si>
+  <si>
+    <t>10,9</t>
+  </si>
+  <si>
+    <t>15 May 2026</t>
   </si>
 </sst>
 </file>
@@ -8236,21 +8242,57 @@
       <c r="AF83" s="2"/>
     </row>
     <row r="84" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A84" s="2"/>
-      <c r="B84" s="2"/>
-      <c r="C84" s="2"/>
-      <c r="D84" s="2"/>
-      <c r="E84" s="2"/>
-      <c r="F84" s="2"/>
-      <c r="G84" s="2"/>
-      <c r="H84" s="2"/>
-      <c r="I84" s="2"/>
-      <c r="J84" s="2"/>
-      <c r="K84" s="2"/>
-      <c r="L84" s="2"/>
-      <c r="M84" s="2"/>
-      <c r="N84" s="2"/>
-      <c r="O84" s="2"/>
+      <c r="A84" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H84" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="I84" s="2">
+        <v>-4</v>
+      </c>
+      <c r="J84" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K84" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L84" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M84" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N84" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O84" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P84" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q84" s="4" t="s">
+        <v>54</v>
+      </c>
       <c r="R84" s="2"/>
       <c r="S84" s="2"/>
       <c r="T84" s="2"/>

</xml_diff>

<commit_message>
Add new temporary file for Dataset Analisis Trading.xlsx
</commit_message>
<xml_diff>
--- a/Dataset Analisis Trading.xlsx
+++ b/Dataset Analisis Trading.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\Fibpath Analyzer\fibpath-analyzer-v3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19FCDB43-0DE2-40BA-8ED9-863C880915C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C49EE510-BC86-4DA1-8E91-E848575CDE5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="13403" windowWidth="21795" windowHeight="12975" xr2:uid="{0FBFC3C1-39E9-48C7-94FA-7929923CC50D}"/>
   </bookViews>
@@ -8293,12 +8293,24 @@
       <c r="Q84" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="R84" s="2"/>
-      <c r="S84" s="2"/>
-      <c r="T84" s="2"/>
-      <c r="U84" s="2"/>
-      <c r="V84" s="2"/>
-      <c r="W84" s="2"/>
+      <c r="R84" s="2">
+        <v>0</v>
+      </c>
+      <c r="S84" s="2">
+        <v>1</v>
+      </c>
+      <c r="T84" s="2">
+        <v>0</v>
+      </c>
+      <c r="U84" s="2">
+        <v>1</v>
+      </c>
+      <c r="V84" s="2">
+        <v>0</v>
+      </c>
+      <c r="W84" s="2">
+        <v>2</v>
+      </c>
       <c r="X84" s="2"/>
       <c r="Y84" s="2"/>
       <c r="Z84" s="2"/>

</xml_diff>

<commit_message>
Add initial ASUS data to ETH spreadsheet
</commit_message>
<xml_diff>
--- a/Dataset Analisis Trading.xlsx
+++ b/Dataset Analisis Trading.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\Fibpath Analyzer\fibpath-analyzer-v3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C49EE510-BC86-4DA1-8E91-E848575CDE5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3497A21-2F9C-4420-ADF5-1B3F024D602F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="13403" windowWidth="21795" windowHeight="12975" xr2:uid="{0FBFC3C1-39E9-48C7-94FA-7929923CC50D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1355" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1371" uniqueCount="170">
   <si>
     <t>Trend</t>
   </si>
@@ -538,6 +538,12 @@
   </si>
   <si>
     <t>15 May 2026</t>
+  </si>
+  <si>
+    <t>24,1</t>
+  </si>
+  <si>
+    <t>14 May 2026</t>
   </si>
 </sst>
 </file>
@@ -3925,73 +3931,73 @@
     </row>
     <row r="30" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>99</v>
+        <v>33</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>95</v>
+        <v>114</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>100</v>
+        <v>168</v>
       </c>
       <c r="I30" s="2">
-        <v>-3</v>
+        <v>3</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K30" s="2" t="s">
         <v>38</v>
       </c>
       <c r="L30" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M30" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M30" s="2" t="s">
+      <c r="N30" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="N30" s="2" t="s">
+      <c r="O30" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="O30" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="P30" s="3" t="s">
-        <v>101</v>
+      <c r="P30" s="4" t="s">
+        <v>169</v>
       </c>
       <c r="Q30" s="4" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
       <c r="R30" s="2">
+        <v>0</v>
+      </c>
+      <c r="S30" s="2">
         <v>1</v>
       </c>
-      <c r="S30" s="2">
+      <c r="T30" s="2">
+        <v>0</v>
+      </c>
+      <c r="U30" s="2">
         <v>2</v>
       </c>
-      <c r="T30" s="2">
+      <c r="V30" s="2">
+        <v>0</v>
+      </c>
+      <c r="W30" s="2">
         <v>3</v>
-      </c>
-      <c r="U30" s="2">
-        <v>0</v>
-      </c>
-      <c r="V30" s="2">
-        <v>4</v>
-      </c>
-      <c r="W30" s="2">
-        <v>0</v>
       </c>
       <c r="X30" s="2"/>
       <c r="Y30" s="2"/>
@@ -4005,73 +4011,73 @@
     </row>
     <row r="31" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="G31" s="2" t="s">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>104</v>
+        <v>166</v>
       </c>
       <c r="I31" s="2">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K31" s="2" t="s">
         <v>38</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M31" s="2" t="s">
         <v>38</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O31" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P31" s="3" t="s">
-        <v>101</v>
+      <c r="P31" s="4" t="s">
+        <v>167</v>
       </c>
       <c r="Q31" s="4" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="R31" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S31" s="2">
         <v>1</v>
       </c>
       <c r="T31" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U31" s="2">
         <v>1</v>
       </c>
       <c r="V31" s="2">
+        <v>0</v>
+      </c>
+      <c r="W31" s="2">
         <v>2</v>
-      </c>
-      <c r="W31" s="2">
-        <v>1</v>
       </c>
       <c r="X31" s="2"/>
       <c r="Y31" s="2"/>
@@ -4091,13 +4097,13 @@
         <v>99</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>79</v>
@@ -4106,7 +4112,7 @@
         <v>79</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="I32" s="2">
         <v>-3</v>
@@ -4121,37 +4127,37 @@
         <v>38</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N32" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O32" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P32" s="3" t="s">
         <v>101</v>
       </c>
       <c r="Q32" s="4" t="s">
-        <v>44</v>
+        <v>102</v>
       </c>
       <c r="R32" s="2">
         <v>1</v>
       </c>
       <c r="S32" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T32" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U32" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V32" s="2">
         <v>4</v>
       </c>
       <c r="W32" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X32" s="2"/>
       <c r="Y32" s="2"/>
@@ -4174,22 +4180,22 @@
         <v>99</v>
       </c>
       <c r="D33" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>48</v>
-      </c>
       <c r="F33" s="2" t="s">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I33" s="2">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="J33" s="2" t="s">
         <v>38</v>
@@ -4207,31 +4213,31 @@
         <v>38</v>
       </c>
       <c r="O33" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P33" s="3" t="s">
         <v>101</v>
       </c>
       <c r="Q33" s="4" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="R33" s="2">
         <v>1</v>
       </c>
       <c r="S33" s="2">
+        <v>1</v>
+      </c>
+      <c r="T33" s="2">
         <v>2</v>
       </c>
-      <c r="T33" s="2">
-        <v>4</v>
-      </c>
       <c r="U33" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V33" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W33" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X33" s="2"/>
       <c r="Y33" s="2"/>
@@ -4254,10 +4260,10 @@
         <v>99</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>35</v>
+        <v>103</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>79</v>
@@ -4266,10 +4272,10 @@
         <v>79</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I34" s="2">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="J34" s="2" t="s">
         <v>38</v>
@@ -4281,37 +4287,37 @@
         <v>38</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N34" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O34" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P34" s="3" t="s">
         <v>101</v>
       </c>
       <c r="Q34" s="4" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="R34" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S34" s="2">
         <v>1</v>
       </c>
       <c r="T34" s="2">
+        <v>1</v>
+      </c>
+      <c r="U34" s="2">
         <v>2</v>
       </c>
-      <c r="U34" s="2">
-        <v>0</v>
-      </c>
       <c r="V34" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W34" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X34" s="2"/>
       <c r="Y34" s="2"/>
@@ -4334,10 +4340,10 @@
         <v>99</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>34</v>
+        <v>96</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>79</v>
@@ -4346,10 +4352,10 @@
         <v>79</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I35" s="2">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>38</v>
@@ -4373,7 +4379,7 @@
         <v>101</v>
       </c>
       <c r="Q35" s="4" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="R35" s="2">
         <v>1</v>
@@ -4382,7 +4388,7 @@
         <v>2</v>
       </c>
       <c r="T35" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U35" s="2">
         <v>3</v>
@@ -4414,10 +4420,10 @@
         <v>99</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="F36" s="2" t="s">
         <v>79</v>
@@ -4426,10 +4432,10 @@
         <v>79</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="I36" s="2">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="J36" s="2" t="s">
         <v>38</v>
@@ -4441,19 +4447,19 @@
         <v>38</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N36" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O36" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P36" s="3" t="s">
         <v>101</v>
       </c>
       <c r="Q36" s="4" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="R36" s="2">
         <v>2</v>
@@ -4465,13 +4471,13 @@
         <v>2</v>
       </c>
       <c r="U36" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V36" s="2">
         <v>2</v>
       </c>
       <c r="W36" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X36" s="2"/>
       <c r="Y36" s="2"/>
@@ -4494,10 +4500,10 @@
         <v>99</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>79</v>
@@ -4506,10 +4512,10 @@
         <v>79</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I37" s="2">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="J37" s="2" t="s">
         <v>38</v>
@@ -4527,31 +4533,31 @@
         <v>38</v>
       </c>
       <c r="O37" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P37" s="3" t="s">
         <v>101</v>
       </c>
       <c r="Q37" s="4" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="R37" s="2">
+        <v>1</v>
+      </c>
+      <c r="S37" s="2">
         <v>2</v>
       </c>
-      <c r="S37" s="2">
+      <c r="T37" s="2">
         <v>1</v>
       </c>
-      <c r="T37" s="2">
-        <v>2</v>
-      </c>
       <c r="U37" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V37" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W37" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X37" s="2"/>
       <c r="Y37" s="2"/>
@@ -4574,10 +4580,10 @@
         <v>99</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>79</v>
@@ -4586,7 +4592,7 @@
         <v>79</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I38" s="2">
         <v>-3</v>
@@ -4607,13 +4613,13 @@
         <v>38</v>
       </c>
       <c r="O38" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P38" s="3" t="s">
         <v>101</v>
       </c>
       <c r="Q38" s="4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="R38" s="2">
         <v>2</v>
@@ -4631,7 +4637,7 @@
         <v>2</v>
       </c>
       <c r="W38" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X38" s="2"/>
       <c r="Y38" s="2"/>
@@ -4648,16 +4654,16 @@
         <v>79</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>99</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>79</v>
@@ -4666,52 +4672,52 @@
         <v>79</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I39" s="2">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="J39" s="2" t="s">
         <v>38</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L39" s="2" t="s">
         <v>38</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N39" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O39" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P39" s="3" t="s">
         <v>101</v>
       </c>
       <c r="Q39" s="4" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="R39" s="2">
+        <v>2</v>
+      </c>
+      <c r="S39" s="2">
         <v>1</v>
       </c>
-      <c r="S39" s="2">
-        <v>0</v>
-      </c>
       <c r="T39" s="2">
+        <v>2</v>
+      </c>
+      <c r="U39" s="2">
         <v>1</v>
       </c>
-      <c r="U39" s="2">
-        <v>0</v>
-      </c>
       <c r="V39" s="2">
+        <v>2</v>
+      </c>
+      <c r="W39" s="2">
         <v>1</v>
-      </c>
-      <c r="W39" s="2">
-        <v>0</v>
       </c>
       <c r="X39" s="2"/>
       <c r="Y39" s="2"/>
@@ -4728,40 +4734,40 @@
         <v>79</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="I40" s="2">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="J40" s="2" t="s">
         <v>38</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L40" s="2" t="s">
         <v>38</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N40" s="2" t="s">
         <v>38</v>
@@ -4773,19 +4779,19 @@
         <v>101</v>
       </c>
       <c r="Q40" s="4" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="R40" s="2">
+        <v>2</v>
+      </c>
+      <c r="S40" s="2">
         <v>1</v>
       </c>
-      <c r="S40" s="2">
-        <v>0</v>
-      </c>
       <c r="T40" s="2">
+        <v>2</v>
+      </c>
+      <c r="U40" s="2">
         <v>1</v>
-      </c>
-      <c r="U40" s="2">
-        <v>0</v>
       </c>
       <c r="V40" s="2">
         <v>2</v>
@@ -4805,37 +4811,37 @@
     </row>
     <row r="41" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>114</v>
+        <v>78</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="I41" s="2">
-        <v>5</v>
+        <v>-5</v>
       </c>
       <c r="J41" s="2" t="s">
         <v>38</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>38</v>
@@ -4844,7 +4850,7 @@
         <v>39</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="O41" s="2" t="s">
         <v>39</v>
@@ -4853,22 +4859,22 @@
         <v>101</v>
       </c>
       <c r="Q41" s="4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="R41" s="2">
         <v>1</v>
       </c>
       <c r="S41" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T41" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U41" s="2">
         <v>0</v>
       </c>
       <c r="V41" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W41" s="2">
         <v>0</v>
@@ -4885,73 +4891,73 @@
     </row>
     <row r="42" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>33</v>
+        <v>114</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>114</v>
+        <v>78</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="I42" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J42" s="2" t="s">
         <v>38</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L42" s="2" t="s">
         <v>38</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N42" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O42" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P42" s="3" t="s">
         <v>101</v>
       </c>
       <c r="Q42" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="R42" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S42" s="2">
+        <v>0</v>
+      </c>
+      <c r="T42" s="2">
         <v>1</v>
       </c>
-      <c r="T42" s="2">
-        <v>5</v>
-      </c>
       <c r="U42" s="2">
+        <v>0</v>
+      </c>
+      <c r="V42" s="2">
         <v>2</v>
       </c>
-      <c r="V42" s="2">
-        <v>6</v>
-      </c>
       <c r="W42" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X42" s="2"/>
       <c r="Y42" s="2"/>
@@ -4968,25 +4974,25 @@
         <v>32</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>33</v>
+        <v>114</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>33</v>
+        <v>114</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="F43" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I43" s="2">
         <v>5</v>
@@ -5001,37 +5007,37 @@
         <v>38</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O43" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P43" s="3" t="s">
         <v>101</v>
       </c>
       <c r="Q43" s="4" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="R43" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S43" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T43" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U43" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V43" s="2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W43" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X43" s="2"/>
       <c r="Y43" s="2"/>
@@ -5051,13 +5057,13 @@
         <v>33</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>33</v>
+        <v>114</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="F44" s="2" t="s">
         <v>32</v>
@@ -5066,7 +5072,7 @@
         <v>32</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I44" s="2">
         <v>5</v>
@@ -5084,7 +5090,7 @@
         <v>38</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="O44" s="2" t="s">
         <v>38</v>
@@ -5093,22 +5099,22 @@
         <v>101</v>
       </c>
       <c r="Q44" s="4" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="R44" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S44" s="2">
         <v>1</v>
       </c>
       <c r="T44" s="2">
+        <v>5</v>
+      </c>
+      <c r="U44" s="2">
         <v>2</v>
       </c>
-      <c r="U44" s="2">
-        <v>3</v>
-      </c>
       <c r="V44" s="2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="W44" s="2">
         <v>3</v>
@@ -5134,10 +5140,10 @@
         <v>33</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>96</v>
+        <v>45</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>32</v>
@@ -5146,7 +5152,7 @@
         <v>32</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I45" s="2">
         <v>5</v>
@@ -5158,13 +5164,13 @@
         <v>38</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M45" s="2" t="s">
         <v>38</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="O45" s="2" t="s">
         <v>38</v>
@@ -5173,25 +5179,25 @@
         <v>101</v>
       </c>
       <c r="Q45" s="4" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="R45" s="2">
+        <v>4</v>
+      </c>
+      <c r="S45" s="2">
         <v>1</v>
       </c>
-      <c r="S45" s="2">
+      <c r="T45" s="2">
+        <v>5</v>
+      </c>
+      <c r="U45" s="2">
         <v>2</v>
       </c>
-      <c r="T45" s="2">
-        <v>0</v>
-      </c>
-      <c r="U45" s="2">
+      <c r="V45" s="2">
+        <v>6</v>
+      </c>
+      <c r="W45" s="2">
         <v>3</v>
-      </c>
-      <c r="V45" s="2">
-        <v>0</v>
-      </c>
-      <c r="W45" s="2">
-        <v>4</v>
       </c>
       <c r="X45" s="2"/>
       <c r="Y45" s="2"/>
@@ -5214,10 +5220,10 @@
         <v>33</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>96</v>
+        <v>45</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>32</v>
@@ -5226,7 +5232,7 @@
         <v>32</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I46" s="2">
         <v>5</v>
@@ -5253,25 +5259,25 @@
         <v>101</v>
       </c>
       <c r="Q46" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="R46" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S46" s="2">
         <v>1</v>
       </c>
       <c r="T46" s="2">
+        <v>2</v>
+      </c>
+      <c r="U46" s="2">
         <v>3</v>
-      </c>
-      <c r="U46" s="2">
-        <v>4</v>
       </c>
       <c r="V46" s="2">
         <v>0</v>
       </c>
       <c r="W46" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="X46" s="2"/>
       <c r="Y46" s="2"/>
@@ -5294,10 +5300,10 @@
         <v>33</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="F47" s="2" t="s">
         <v>32</v>
@@ -5306,7 +5312,7 @@
         <v>32</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I47" s="2">
         <v>5</v>
@@ -5318,22 +5324,22 @@
         <v>38</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M47" s="2" t="s">
         <v>38</v>
       </c>
       <c r="N47" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O47" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="O47" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="P47" s="3" t="s">
         <v>101</v>
       </c>
       <c r="Q47" s="4" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="R47" s="2">
         <v>1</v>
@@ -5342,16 +5348,16 @@
         <v>2</v>
       </c>
       <c r="T47" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U47" s="2">
         <v>3</v>
       </c>
       <c r="V47" s="2">
+        <v>0</v>
+      </c>
+      <c r="W47" s="2">
         <v>4</v>
-      </c>
-      <c r="W47" s="2">
-        <v>0</v>
       </c>
       <c r="X47" s="2"/>
       <c r="Y47" s="2"/>
@@ -5374,10 +5380,10 @@
         <v>33</v>
       </c>
       <c r="D48" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E48" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>72</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>32</v>
@@ -5386,19 +5392,19 @@
         <v>32</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I48" s="2">
         <v>5</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K48" s="2" t="s">
         <v>38</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M48" s="2" t="s">
         <v>38</v>
@@ -5413,25 +5419,25 @@
         <v>101</v>
       </c>
       <c r="Q48" s="4" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="R48" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S48" s="2">
         <v>1</v>
       </c>
       <c r="T48" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U48" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V48" s="2">
         <v>0</v>
       </c>
       <c r="W48" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="X48" s="2"/>
       <c r="Y48" s="2"/>
@@ -5454,10 +5460,10 @@
         <v>33</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>96</v>
+        <v>62</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>32</v>
@@ -5466,52 +5472,52 @@
         <v>32</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I49" s="2">
         <v>5</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K49" s="2" t="s">
         <v>38</v>
       </c>
       <c r="L49" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M49" s="2" t="s">
         <v>38</v>
       </c>
       <c r="N49" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O49" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="O49" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="P49" s="3" t="s">
         <v>101</v>
       </c>
       <c r="Q49" s="4" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="R49" s="2">
+        <v>1</v>
+      </c>
+      <c r="S49" s="2">
+        <v>2</v>
+      </c>
+      <c r="T49" s="2">
+        <v>1</v>
+      </c>
+      <c r="U49" s="2">
+        <v>3</v>
+      </c>
+      <c r="V49" s="2">
+        <v>4</v>
+      </c>
+      <c r="W49" s="2">
         <v>0</v>
-      </c>
-      <c r="S49" s="2">
-        <v>1</v>
-      </c>
-      <c r="T49" s="2">
-        <v>0</v>
-      </c>
-      <c r="U49" s="2">
-        <v>2</v>
-      </c>
-      <c r="V49" s="2">
-        <v>0</v>
-      </c>
-      <c r="W49" s="2">
-        <v>3</v>
       </c>
       <c r="X49" s="2"/>
       <c r="Y49" s="2"/>
@@ -5525,31 +5531,31 @@
     </row>
     <row r="50" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>90</v>
+        <v>33</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D50" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E50" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E50" s="1" t="s">
-        <v>103</v>
-      </c>
       <c r="F50" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="H50" s="1" t="s">
-        <v>158</v>
+        <v>32</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>123</v>
       </c>
       <c r="I50" s="2">
-        <v>-3</v>
+        <v>5</v>
       </c>
       <c r="J50" s="2" t="s">
         <v>39</v>
@@ -5569,11 +5575,11 @@
       <c r="O50" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P50" s="4" t="s">
-        <v>157</v>
+      <c r="P50" s="3" t="s">
+        <v>101</v>
       </c>
       <c r="Q50" s="4" t="s">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="R50" s="2">
         <v>0</v>
@@ -5626,51 +5632,53 @@
         <v>32</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>159</v>
+        <v>124</v>
       </c>
       <c r="I51" s="2">
         <v>5</v>
       </c>
       <c r="J51" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K51" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K51" s="2" t="s">
+      <c r="L51" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="L51" s="2" t="s">
+      <c r="M51" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M51" s="2" t="s">
+      <c r="N51" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="N51" s="2" t="s">
+      <c r="O51" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="O51" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="P51" s="4" t="s">
-        <v>160</v>
+      <c r="P51" s="3" t="s">
+        <v>101</v>
       </c>
       <c r="Q51" s="4" t="s">
-        <v>81</v>
+        <v>98</v>
       </c>
       <c r="R51" s="2">
+        <v>0</v>
+      </c>
+      <c r="S51" s="2">
         <v>1</v>
       </c>
-      <c r="S51" s="2">
+      <c r="T51" s="2">
         <v>0</v>
       </c>
-      <c r="T51" s="2">
-        <v>1</v>
-      </c>
       <c r="U51" s="2">
+        <v>2</v>
+      </c>
+      <c r="V51" s="2">
         <v>0</v>
       </c>
-      <c r="V51" s="2">
-        <v>1</v>
-      </c>
-      <c r="W51" s="2"/>
+      <c r="W51" s="2">
+        <v>3</v>
+      </c>
       <c r="X51" s="2"/>
       <c r="Y51" s="2"/>
       <c r="Z51" s="2"/>
@@ -5683,34 +5691,34 @@
     </row>
     <row r="52" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>33</v>
+        <v>90</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>59</v>
+        <v>90</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>103</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H52" s="2" t="s">
-        <v>125</v>
+        <v>79</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>158</v>
       </c>
       <c r="I52" s="2">
-        <v>5</v>
+        <v>-3</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K52" s="2" t="s">
         <v>38</v>
@@ -5727,14 +5735,14 @@
       <c r="O52" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P52" s="3" t="s">
-        <v>126</v>
+      <c r="P52" s="4" t="s">
+        <v>157</v>
       </c>
       <c r="Q52" s="4" t="s">
-        <v>102</v>
+        <v>56</v>
       </c>
       <c r="R52" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S52" s="2">
         <v>1</v>
@@ -5743,7 +5751,7 @@
         <v>0</v>
       </c>
       <c r="U52" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V52" s="2">
         <v>0</v>
@@ -5766,7 +5774,7 @@
         <v>32</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>33</v>
@@ -5784,53 +5792,51 @@
         <v>32</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>127</v>
+        <v>159</v>
       </c>
       <c r="I53" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J53" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K53" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="K53" s="2" t="s">
+      <c r="L53" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="L53" s="2" t="s">
+      <c r="M53" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="M53" s="2" t="s">
+      <c r="N53" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="N53" s="2" t="s">
+      <c r="O53" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="O53" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="P53" s="3" t="s">
-        <v>126</v>
+      <c r="P53" s="4" t="s">
+        <v>160</v>
       </c>
       <c r="Q53" s="4" t="s">
-        <v>41</v>
+        <v>81</v>
       </c>
       <c r="R53" s="2">
+        <v>1</v>
+      </c>
+      <c r="S53" s="2">
         <v>0</v>
       </c>
-      <c r="S53" s="2">
+      <c r="T53" s="2">
         <v>1</v>
       </c>
-      <c r="T53" s="2">
+      <c r="U53" s="2">
         <v>0</v>
       </c>
-      <c r="U53" s="2">
-        <v>2</v>
-      </c>
       <c r="V53" s="2">
-        <v>0</v>
-      </c>
-      <c r="W53" s="2">
-        <v>3</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="W53" s="2"/>
       <c r="X53" s="2"/>
       <c r="Y53" s="2"/>
       <c r="Z53" s="2"/>
@@ -5846,13 +5852,13 @@
         <v>32</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>59</v>
@@ -5864,13 +5870,13 @@
         <v>32</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I54" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K54" s="2" t="s">
         <v>38</v>
@@ -5891,10 +5897,10 @@
         <v>126</v>
       </c>
       <c r="Q54" s="4" t="s">
-        <v>44</v>
+        <v>102</v>
       </c>
       <c r="R54" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S54" s="2">
         <v>1</v>
@@ -5909,7 +5915,7 @@
         <v>0</v>
       </c>
       <c r="W54" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X54" s="2"/>
       <c r="Y54" s="2"/>
@@ -5929,13 +5935,13 @@
         <v>51</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>32</v>
@@ -5944,13 +5950,13 @@
         <v>32</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I55" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K55" s="2" t="s">
         <v>38</v>
@@ -5971,10 +5977,10 @@
         <v>126</v>
       </c>
       <c r="Q55" s="4" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="R55" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S55" s="2">
         <v>1</v>
@@ -5983,13 +5989,13 @@
         <v>0</v>
       </c>
       <c r="U55" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V55" s="2">
         <v>0</v>
       </c>
       <c r="W55" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X55" s="2"/>
       <c r="Y55" s="2"/>
@@ -6012,10 +6018,10 @@
         <v>51</v>
       </c>
       <c r="D56" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E56" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>45</v>
       </c>
       <c r="F56" s="2" t="s">
         <v>32</v>
@@ -6024,13 +6030,13 @@
         <v>32</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I56" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K56" s="2" t="s">
         <v>38</v>
@@ -6051,10 +6057,10 @@
         <v>126</v>
       </c>
       <c r="Q56" s="4" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="R56" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S56" s="2">
         <v>1</v>
@@ -6092,22 +6098,22 @@
         <v>51</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I57" s="2">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="J57" s="2" t="s">
         <v>38</v>
@@ -6116,13 +6122,13 @@
         <v>38</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M57" s="2" t="s">
         <v>38</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O57" s="2" t="s">
         <v>38</v>
@@ -6131,22 +6137,22 @@
         <v>126</v>
       </c>
       <c r="Q57" s="4" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="R57" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S57" s="2">
         <v>1</v>
       </c>
       <c r="T57" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="U57" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V57" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="W57" s="2">
         <v>2</v>
@@ -6172,22 +6178,22 @@
         <v>51</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I58" s="2">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="J58" s="2" t="s">
         <v>38</v>
@@ -6211,13 +6217,13 @@
         <v>126</v>
       </c>
       <c r="Q58" s="4" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="R58" s="2">
         <v>1</v>
       </c>
       <c r="S58" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T58" s="2">
         <v>0</v>
@@ -6229,7 +6235,7 @@
         <v>0</v>
       </c>
       <c r="W58" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X58" s="2"/>
       <c r="Y58" s="2"/>
@@ -6252,10 +6258,10 @@
         <v>51</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="F59" s="2" t="s">
         <v>79</v>
@@ -6264,25 +6270,25 @@
         <v>79</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I59" s="2">
         <v>-1</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K59" s="2" t="s">
         <v>38</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M59" s="2" t="s">
         <v>38</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="O59" s="2" t="s">
         <v>38</v>
@@ -6291,25 +6297,25 @@
         <v>126</v>
       </c>
       <c r="Q59" s="4" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="R59" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S59" s="2">
         <v>1</v>
       </c>
       <c r="T59" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U59" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V59" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="W59" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X59" s="2"/>
       <c r="Y59" s="2"/>
@@ -6323,28 +6329,28 @@
     </row>
     <row r="60" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>51</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>59</v>
+        <v>96</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="F60" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I60" s="2">
         <v>-1</v>
@@ -6353,43 +6359,43 @@
         <v>38</v>
       </c>
       <c r="K60" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L60" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="L60" s="2" t="s">
+      <c r="M60" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M60" s="2" t="s">
+      <c r="N60" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="N60" s="2" t="s">
+      <c r="O60" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="O60" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="P60" s="3" t="s">
         <v>126</v>
       </c>
       <c r="Q60" s="4" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="R60" s="2">
         <v>1</v>
       </c>
       <c r="S60" s="2">
+        <v>2</v>
+      </c>
+      <c r="T60" s="2">
         <v>0</v>
       </c>
-      <c r="T60" s="2">
-        <v>1</v>
-      </c>
       <c r="U60" s="2">
+        <v>2</v>
+      </c>
+      <c r="V60" s="2">
         <v>0</v>
       </c>
-      <c r="V60" s="2">
+      <c r="W60" s="2">
         <v>2</v>
-      </c>
-      <c r="W60" s="2">
-        <v>0</v>
       </c>
       <c r="X60" s="2"/>
       <c r="Y60" s="2"/>
@@ -6403,19 +6409,19 @@
     </row>
     <row r="61" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>72</v>
+        <v>45</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>35</v>
+        <v>96</v>
       </c>
       <c r="F61" s="2" t="s">
         <v>79</v>
@@ -6424,25 +6430,25 @@
         <v>79</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I61" s="2">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K61" s="2" t="s">
         <v>38</v>
       </c>
       <c r="L61" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M61" s="2" t="s">
         <v>38</v>
       </c>
       <c r="N61" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O61" s="2" t="s">
         <v>38</v>
@@ -6451,25 +6457,25 @@
         <v>126</v>
       </c>
       <c r="Q61" s="4" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="R61" s="2">
+        <v>0</v>
+      </c>
+      <c r="S61" s="2">
         <v>1</v>
       </c>
-      <c r="S61" s="2">
-        <v>3</v>
-      </c>
       <c r="T61" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U61" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V61" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W61" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="X61" s="2"/>
       <c r="Y61" s="2"/>
@@ -6489,67 +6495,67 @@
         <v>90</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>103</v>
+        <v>59</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="F62" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I62" s="2">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="J62" s="2" t="s">
         <v>38</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L62" s="2" t="s">
         <v>38</v>
       </c>
       <c r="M62" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N62" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O62" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P62" s="3" t="s">
         <v>126</v>
       </c>
       <c r="Q62" s="4" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="R62" s="2">
+        <v>1</v>
+      </c>
+      <c r="S62" s="2">
+        <v>0</v>
+      </c>
+      <c r="T62" s="2">
+        <v>1</v>
+      </c>
+      <c r="U62" s="2">
+        <v>0</v>
+      </c>
+      <c r="V62" s="2">
         <v>2</v>
       </c>
-      <c r="S62" s="2">
-        <v>1</v>
-      </c>
-      <c r="T62" s="2">
-        <v>2</v>
-      </c>
-      <c r="U62" s="2">
-        <v>1</v>
-      </c>
-      <c r="V62" s="2">
-        <v>3</v>
-      </c>
       <c r="W62" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X62" s="2"/>
       <c r="Y62" s="2"/>
@@ -6569,13 +6575,13 @@
         <v>90</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>103</v>
+        <v>35</v>
       </c>
       <c r="F63" s="2" t="s">
         <v>79</v>
@@ -6584,7 +6590,7 @@
         <v>79</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I63" s="2">
         <v>-3</v>
@@ -6599,37 +6605,37 @@
         <v>38</v>
       </c>
       <c r="M63" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N63" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O63" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P63" s="3" t="s">
         <v>126</v>
       </c>
       <c r="Q63" s="4" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="R63" s="2">
         <v>1</v>
       </c>
       <c r="S63" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T63" s="2">
         <v>2</v>
       </c>
       <c r="U63" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="V63" s="2">
         <v>2</v>
       </c>
       <c r="W63" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X63" s="2"/>
       <c r="Y63" s="2"/>
@@ -6646,16 +6652,16 @@
         <v>79</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>90</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>34</v>
+        <v>103</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="F64" s="2" t="s">
         <v>79</v>
@@ -6664,52 +6670,52 @@
         <v>79</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I64" s="2">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="J64" s="2" t="s">
         <v>38</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L64" s="2" t="s">
         <v>38</v>
       </c>
       <c r="M64" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N64" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O64" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P64" s="3" t="s">
         <v>126</v>
       </c>
       <c r="Q64" s="4" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="R64" s="2">
+        <v>2</v>
+      </c>
+      <c r="S64" s="2">
         <v>1</v>
       </c>
-      <c r="S64" s="2">
-        <v>0</v>
-      </c>
       <c r="T64" s="2">
+        <v>2</v>
+      </c>
+      <c r="U64" s="2">
         <v>1</v>
       </c>
-      <c r="U64" s="2">
-        <v>0</v>
-      </c>
       <c r="V64" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W64" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X64" s="2"/>
       <c r="Y64" s="2"/>
@@ -6726,25 +6732,25 @@
         <v>79</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>34</v>
+        <v>103</v>
       </c>
       <c r="F65" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="I65" s="2">
         <v>-3</v>
@@ -6759,7 +6765,7 @@
         <v>38</v>
       </c>
       <c r="M65" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N65" s="2" t="s">
         <v>38</v>
@@ -6771,22 +6777,22 @@
         <v>126</v>
       </c>
       <c r="Q65" s="4" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="R65" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S65" s="2">
         <v>1</v>
       </c>
       <c r="T65" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U65" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V65" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="W65" s="2">
         <v>0</v>
@@ -6806,16 +6812,16 @@
         <v>79</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F66" s="2" t="s">
         <v>79</v>
@@ -6824,52 +6830,52 @@
         <v>79</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="I66" s="2">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="J66" s="2" t="s">
         <v>38</v>
       </c>
       <c r="K66" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L66" s="2" t="s">
         <v>38</v>
       </c>
       <c r="M66" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N66" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O66" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P66" s="3" t="s">
         <v>126</v>
       </c>
       <c r="Q66" s="4" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="R66" s="2">
+        <v>1</v>
+      </c>
+      <c r="S66" s="2">
+        <v>0</v>
+      </c>
+      <c r="T66" s="2">
+        <v>1</v>
+      </c>
+      <c r="U66" s="2">
+        <v>0</v>
+      </c>
+      <c r="V66" s="2">
         <v>2</v>
       </c>
-      <c r="S66" s="2">
-        <v>1</v>
-      </c>
-      <c r="T66" s="2">
-        <v>2</v>
-      </c>
-      <c r="U66" s="2">
-        <v>1</v>
-      </c>
-      <c r="V66" s="2">
-        <v>4</v>
-      </c>
       <c r="W66" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X66" s="2"/>
       <c r="Y66" s="2"/>
@@ -6886,25 +6892,25 @@
         <v>79</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="F67" s="2" t="s">
         <v>79</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="H67" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I67" s="2">
         <v>-3</v>
@@ -6931,19 +6937,19 @@
         <v>126</v>
       </c>
       <c r="Q67" s="4" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="R67" s="2">
+        <v>2</v>
+      </c>
+      <c r="S67" s="2">
         <v>1</v>
       </c>
-      <c r="S67" s="2">
+      <c r="T67" s="2">
+        <v>4</v>
+      </c>
+      <c r="U67" s="2">
         <v>3</v>
-      </c>
-      <c r="T67" s="2">
-        <v>2</v>
-      </c>
-      <c r="U67" s="2">
-        <v>4</v>
       </c>
       <c r="V67" s="2">
         <v>5</v>
@@ -6972,22 +6978,22 @@
         <v>99</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>96</v>
+        <v>62</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I68" s="2">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="J68" s="2" t="s">
         <v>38</v>
@@ -7005,31 +7011,31 @@
         <v>38</v>
       </c>
       <c r="O68" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P68" s="3" t="s">
         <v>126</v>
       </c>
       <c r="Q68" s="4" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="R68" s="2">
+        <v>2</v>
+      </c>
+      <c r="S68" s="2">
         <v>1</v>
       </c>
-      <c r="S68" s="2">
+      <c r="T68" s="2">
         <v>2</v>
       </c>
-      <c r="T68" s="2">
-        <v>3</v>
-      </c>
       <c r="U68" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V68" s="2">
         <v>4</v>
       </c>
       <c r="W68" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X68" s="2"/>
       <c r="Y68" s="2"/>
@@ -7046,16 +7052,16 @@
         <v>79</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>45</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="F69" s="2" t="s">
         <v>79</v>
@@ -7064,22 +7070,22 @@
         <v>79</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="I69" s="2">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="J69" s="2" t="s">
         <v>38</v>
       </c>
       <c r="K69" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L69" s="2" t="s">
         <v>38</v>
       </c>
       <c r="M69" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N69" s="2" t="s">
         <v>38</v>
@@ -7088,25 +7094,25 @@
         <v>39</v>
       </c>
       <c r="P69" s="3" t="s">
-        <v>146</v>
+        <v>126</v>
       </c>
       <c r="Q69" s="4" t="s">
-        <v>47</v>
+        <v>92</v>
       </c>
       <c r="R69" s="2">
         <v>1</v>
       </c>
       <c r="S69" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T69" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U69" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="V69" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W69" s="2">
         <v>0</v>
@@ -7126,40 +7132,40 @@
         <v>79</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>71</v>
+        <v>99</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>71</v>
+        <v>99</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I70" s="2">
-        <v>-4</v>
+        <v>1</v>
       </c>
       <c r="J70" s="2" t="s">
         <v>38</v>
       </c>
       <c r="K70" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L70" s="2" t="s">
         <v>38</v>
       </c>
       <c r="M70" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N70" s="2" t="s">
         <v>38</v>
@@ -7168,25 +7174,25 @@
         <v>39</v>
       </c>
       <c r="P70" s="3" t="s">
-        <v>146</v>
+        <v>126</v>
       </c>
       <c r="Q70" s="4" t="s">
-        <v>54</v>
+        <v>94</v>
       </c>
       <c r="R70" s="2">
         <v>1</v>
       </c>
       <c r="S70" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T70" s="2">
+        <v>3</v>
+      </c>
+      <c r="U70" s="2">
         <v>2</v>
       </c>
-      <c r="U70" s="2">
-        <v>0</v>
-      </c>
       <c r="V70" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W70" s="2">
         <v>0</v>
@@ -7206,16 +7212,16 @@
         <v>79</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>71</v>
+        <v>114</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>71</v>
+        <v>114</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>72</v>
+        <v>45</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="F71" s="2" t="s">
         <v>79</v>
@@ -7224,10 +7230,10 @@
         <v>79</v>
       </c>
       <c r="H71" s="2" t="s">
-        <v>46</v>
+        <v>145</v>
       </c>
       <c r="I71" s="2">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="J71" s="2" t="s">
         <v>38</v>
@@ -7251,7 +7257,7 @@
         <v>146</v>
       </c>
       <c r="Q71" s="4" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="R71" s="2">
         <v>1</v>
@@ -7266,7 +7272,7 @@
         <v>0</v>
       </c>
       <c r="V71" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W71" s="2">
         <v>0</v>
@@ -7286,28 +7292,28 @@
         <v>79</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>114</v>
+        <v>71</v>
       </c>
       <c r="C72" s="2" t="s">
         <v>71</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I72" s="2">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="J72" s="2" t="s">
         <v>38</v>
@@ -7331,7 +7337,7 @@
         <v>146</v>
       </c>
       <c r="Q72" s="4" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="R72" s="2">
         <v>1</v>
@@ -7340,7 +7346,7 @@
         <v>0</v>
       </c>
       <c r="T72" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U72" s="2">
         <v>0</v>
@@ -7363,31 +7369,31 @@
     </row>
     <row r="73" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A73" s="2" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>114</v>
+        <v>71</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>114</v>
+        <v>71</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>149</v>
+        <v>46</v>
       </c>
       <c r="I73" s="2">
-        <v>5</v>
+        <v>-2</v>
       </c>
       <c r="J73" s="2" t="s">
         <v>38</v>
@@ -7402,7 +7408,7 @@
         <v>39</v>
       </c>
       <c r="N73" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="O73" s="2" t="s">
         <v>39</v>
@@ -7411,7 +7417,7 @@
         <v>146</v>
       </c>
       <c r="Q73" s="4" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="R73" s="2">
         <v>1</v>
@@ -7420,13 +7426,13 @@
         <v>0</v>
       </c>
       <c r="T73" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U73" s="2">
         <v>0</v>
       </c>
       <c r="V73" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W73" s="2">
         <v>0</v>
@@ -7443,19 +7449,19 @@
     </row>
     <row r="74" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A74" s="2" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>33</v>
+        <v>114</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>114</v>
+        <v>71</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="F74" s="2" t="s">
         <v>32</v>
@@ -7464,22 +7470,22 @@
         <v>32</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="I74" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J74" s="2" t="s">
         <v>38</v>
       </c>
       <c r="K74" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L74" s="2" t="s">
         <v>38</v>
       </c>
       <c r="M74" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N74" s="2" t="s">
         <v>38</v>
@@ -7491,22 +7497,22 @@
         <v>146</v>
       </c>
       <c r="Q74" s="4" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="R74" s="2">
         <v>1</v>
       </c>
       <c r="S74" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T74" s="2">
         <v>1</v>
       </c>
       <c r="U74" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V74" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W74" s="2">
         <v>0</v>
@@ -7526,25 +7532,25 @@
         <v>32</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>33</v>
+        <v>114</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>33</v>
+        <v>114</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="F75" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="I75" s="2">
         <v>5</v>
@@ -7553,7 +7559,7 @@
         <v>38</v>
       </c>
       <c r="K75" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L75" s="2" t="s">
         <v>38</v>
@@ -7562,7 +7568,7 @@
         <v>39</v>
       </c>
       <c r="N75" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O75" s="2" t="s">
         <v>39</v>
@@ -7571,13 +7577,13 @@
         <v>146</v>
       </c>
       <c r="Q75" s="4" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="R75" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S75" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T75" s="2">
         <v>2</v>
@@ -7586,7 +7592,7 @@
         <v>0</v>
       </c>
       <c r="V75" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W75" s="2">
         <v>0</v>
@@ -7609,13 +7615,13 @@
         <v>33</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>33</v>
+        <v>114</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>96</v>
+        <v>42</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F76" s="2" t="s">
         <v>32</v>
@@ -7624,7 +7630,7 @@
         <v>32</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I76" s="2">
         <v>5</v>
@@ -7633,13 +7639,13 @@
         <v>38</v>
       </c>
       <c r="K76" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L76" s="2" t="s">
         <v>38</v>
       </c>
       <c r="M76" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N76" s="2" t="s">
         <v>38</v>
@@ -7651,22 +7657,22 @@
         <v>146</v>
       </c>
       <c r="Q76" s="4" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="R76" s="2">
         <v>1</v>
       </c>
       <c r="S76" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T76" s="2">
         <v>1</v>
       </c>
       <c r="U76" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V76" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W76" s="2">
         <v>0</v>
@@ -7692,19 +7698,19 @@
         <v>33</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>96</v>
+        <v>48</v>
       </c>
       <c r="F77" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="H77" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I77" s="2">
         <v>5</v>
@@ -7725,31 +7731,31 @@
         <v>38</v>
       </c>
       <c r="O77" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P77" s="3" t="s">
         <v>146</v>
       </c>
       <c r="Q77" s="4" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="R77" s="2">
+        <v>2</v>
+      </c>
+      <c r="S77" s="2">
         <v>1</v>
       </c>
-      <c r="S77" s="2">
+      <c r="T77" s="2">
         <v>2</v>
       </c>
-      <c r="T77" s="2">
-        <v>1</v>
-      </c>
       <c r="U77" s="2">
+        <v>0</v>
+      </c>
+      <c r="V77" s="2">
         <v>3</v>
       </c>
-      <c r="V77" s="2">
-        <v>1</v>
-      </c>
       <c r="W77" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X77" s="2"/>
       <c r="Y77" s="2"/>
@@ -7772,19 +7778,19 @@
         <v>33</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>34</v>
+        <v>96</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="F78" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="H78" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="I78" s="2">
         <v>5</v>
@@ -7793,16 +7799,16 @@
         <v>38</v>
       </c>
       <c r="K78" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="L78" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="L78" s="2" t="s">
+      <c r="M78" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="M78" s="2" t="s">
+      <c r="N78" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="N78" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="O78" s="2" t="s">
         <v>39</v>
@@ -7811,22 +7817,22 @@
         <v>146</v>
       </c>
       <c r="Q78" s="4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="R78" s="2">
         <v>1</v>
       </c>
       <c r="S78" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T78" s="2">
+        <v>1</v>
+      </c>
+      <c r="U78" s="2">
         <v>0</v>
       </c>
-      <c r="U78" s="2">
-        <v>3</v>
-      </c>
       <c r="V78" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W78" s="2">
         <v>0</v>
@@ -7852,19 +7858,19 @@
         <v>33</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>34</v>
+        <v>96</v>
       </c>
       <c r="F79" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="H79" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="I79" s="2">
         <v>5</v>
@@ -7876,37 +7882,37 @@
         <v>38</v>
       </c>
       <c r="L79" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M79" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="M79" s="2" t="s">
+      <c r="N79" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="N79" s="2" t="s">
-        <v>39</v>
-      </c>
       <c r="O79" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P79" s="3" t="s">
         <v>146</v>
       </c>
       <c r="Q79" s="4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="R79" s="2">
         <v>1</v>
       </c>
       <c r="S79" s="2">
+        <v>2</v>
+      </c>
+      <c r="T79" s="2">
         <v>1</v>
       </c>
-      <c r="T79" s="2">
-        <v>2</v>
-      </c>
       <c r="U79" s="2">
+        <v>3</v>
+      </c>
+      <c r="V79" s="2">
         <v>1</v>
-      </c>
-      <c r="V79" s="2">
-        <v>3</v>
       </c>
       <c r="W79" s="2">
         <v>4</v>
@@ -7941,10 +7947,10 @@
         <v>32</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="H80" s="2" t="s">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="I80" s="2">
         <v>5</v>
@@ -7956,7 +7962,7 @@
         <v>38</v>
       </c>
       <c r="L80" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M80" s="2" t="s">
         <v>38</v>
@@ -7965,13 +7971,13 @@
         <v>39</v>
       </c>
       <c r="O80" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P80" s="3" t="s">
         <v>146</v>
       </c>
       <c r="Q80" s="4" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="R80" s="2">
         <v>1</v>
@@ -7980,7 +7986,7 @@
         <v>2</v>
       </c>
       <c r="T80" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U80" s="2">
         <v>3</v>
@@ -7989,7 +7995,7 @@
         <v>0</v>
       </c>
       <c r="W80" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X80" s="2"/>
       <c r="Y80" s="2"/>
@@ -8012,7 +8018,7 @@
         <v>33</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>34</v>
@@ -8024,13 +8030,13 @@
         <v>32</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I81" s="2">
         <v>5</v>
       </c>
       <c r="J81" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K81" s="2" t="s">
         <v>38</v>
@@ -8045,31 +8051,31 @@
         <v>39</v>
       </c>
       <c r="O81" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P81" s="3" t="s">
         <v>146</v>
       </c>
       <c r="Q81" s="4" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="R81" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S81" s="2">
         <v>1</v>
       </c>
       <c r="T81" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U81" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V81" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W81" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X81" s="2"/>
       <c r="Y81" s="2"/>
@@ -8092,10 +8098,10 @@
         <v>33</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>59</v>
+        <v>34</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="F82" s="2" t="s">
         <v>32</v>
@@ -8104,19 +8110,19 @@
         <v>32</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="I82" s="2">
         <v>5</v>
       </c>
       <c r="J82" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K82" s="2" t="s">
         <v>38</v>
       </c>
       <c r="L82" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M82" s="2" t="s">
         <v>38</v>
@@ -8131,25 +8137,25 @@
         <v>146</v>
       </c>
       <c r="Q82" s="4" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="R82" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S82" s="2">
+        <v>2</v>
+      </c>
+      <c r="T82" s="2">
         <v>1</v>
       </c>
-      <c r="T82" s="2">
-        <v>0</v>
-      </c>
       <c r="U82" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V82" s="2">
         <v>0</v>
       </c>
       <c r="W82" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X82" s="2"/>
       <c r="Y82" s="2"/>
@@ -8166,16 +8172,16 @@
         <v>32</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F83" s="2" t="s">
         <v>32</v>
@@ -8184,13 +8190,13 @@
         <v>32</v>
       </c>
       <c r="H83" s="2" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="I83" s="2">
         <v>5</v>
       </c>
       <c r="J83" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K83" s="2" t="s">
         <v>38</v>
@@ -8211,10 +8217,10 @@
         <v>146</v>
       </c>
       <c r="Q83" s="4" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="R83" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S83" s="2">
         <v>1</v>
@@ -8229,7 +8235,7 @@
         <v>0</v>
       </c>
       <c r="W83" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="X83" s="2"/>
       <c r="Y83" s="2"/>
@@ -8246,28 +8252,28 @@
         <v>32</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="D84" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="G84" s="2" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="H84" s="2" t="s">
-        <v>166</v>
+        <v>108</v>
       </c>
       <c r="I84" s="2">
-        <v>-4</v>
+        <v>5</v>
       </c>
       <c r="J84" s="2" t="s">
         <v>39</v>
@@ -8287,11 +8293,11 @@
       <c r="O84" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P84" s="4" t="s">
-        <v>167</v>
+      <c r="P84" s="3" t="s">
+        <v>146</v>
       </c>
       <c r="Q84" s="4" t="s">
-        <v>54</v>
+        <v>89</v>
       </c>
       <c r="R84" s="2">
         <v>0</v>
@@ -8303,13 +8309,13 @@
         <v>0</v>
       </c>
       <c r="U84" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V84" s="2">
         <v>0</v>
       </c>
       <c r="W84" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X84" s="2"/>
       <c r="Y84" s="2"/>
@@ -8322,27 +8328,75 @@
       <c r="AF84" s="2"/>
     </row>
     <row r="85" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A85" s="2"/>
-      <c r="B85" s="2"/>
-      <c r="C85" s="2"/>
-      <c r="D85" s="2"/>
-      <c r="E85" s="2"/>
-      <c r="F85" s="2"/>
-      <c r="G85" s="2"/>
-      <c r="H85" s="2"/>
-      <c r="I85" s="2"/>
-      <c r="J85" s="2"/>
-      <c r="K85" s="2"/>
-      <c r="L85" s="2"/>
-      <c r="M85" s="2"/>
-      <c r="N85" s="2"/>
-      <c r="O85" s="2"/>
-      <c r="R85" s="2"/>
-      <c r="S85" s="2"/>
-      <c r="T85" s="2"/>
-      <c r="U85" s="2"/>
-      <c r="V85" s="2"/>
-      <c r="W85" s="2"/>
+      <c r="A85" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H85" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="I85" s="2">
+        <v>5</v>
+      </c>
+      <c r="J85" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K85" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L85" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M85" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N85" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O85" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P85" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q85" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="R85" s="2">
+        <v>3</v>
+      </c>
+      <c r="S85" s="2">
+        <v>1</v>
+      </c>
+      <c r="T85" s="2">
+        <v>0</v>
+      </c>
+      <c r="U85" s="2">
+        <v>2</v>
+      </c>
+      <c r="V85" s="2">
+        <v>0</v>
+      </c>
+      <c r="W85" s="2">
+        <v>4</v>
+      </c>
       <c r="X85" s="2"/>
       <c r="Y85" s="2"/>
       <c r="Z85" s="2"/>

</xml_diff>

<commit_message>
Update trading analysis files and add signal generation script
- Updated model_id in Analisa.ipynb for widget compatibility.
- Modified Dataset Analisis Trading.xlsx and ETH.xlsx files to reflect new data.
- Added new settings.json file to configure permissions for script execution.
- Introduced ETH_signals_14-17May2026.xlsx to store hourly trading signals.
- Created generate_hourly_signals.py script to automate the generation of trading signals for ETH-USD from May 14 to May 17, 2026.
</commit_message>
<xml_diff>
--- a/Dataset Analisis Trading.xlsx
+++ b/Dataset Analisis Trading.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\Fibpath Analyzer\fibpath-analyzer-v3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3497A21-2F9C-4420-ADF5-1B3F024D602F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE7AF8F8-4C4C-43C5-BCC8-20D84CDD570E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="13403" windowWidth="21795" windowHeight="12975" xr2:uid="{0FBFC3C1-39E9-48C7-94FA-7929923CC50D}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{0FBFC3C1-39E9-48C7-94FA-7929923CC50D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1371" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1611" uniqueCount="170">
   <si>
     <t>Trend</t>
   </si>
@@ -592,7 +592,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -608,6 +608,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8408,27 +8411,75 @@
       <c r="AF85" s="2"/>
     </row>
     <row r="86" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A86" s="2"/>
-      <c r="B86" s="2"/>
-      <c r="C86" s="2"/>
-      <c r="D86" s="2"/>
-      <c r="E86" s="2"/>
-      <c r="F86" s="2"/>
-      <c r="G86" s="2"/>
-      <c r="H86" s="2"/>
-      <c r="I86" s="2"/>
-      <c r="J86" s="2"/>
-      <c r="K86" s="2"/>
-      <c r="L86" s="2"/>
-      <c r="M86" s="2"/>
-      <c r="N86" s="2"/>
-      <c r="O86" s="2"/>
-      <c r="R86" s="2"/>
-      <c r="S86" s="2"/>
-      <c r="T86" s="2"/>
-      <c r="U86" s="2"/>
-      <c r="V86" s="2"/>
-      <c r="W86" s="2"/>
+      <c r="A86" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G86" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H86" s="6">
+        <v>23.5</v>
+      </c>
+      <c r="I86" s="6">
+        <v>3</v>
+      </c>
+      <c r="J86" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K86" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L86" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M86" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N86" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O86" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P86" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q86" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="R86" s="2">
+        <v>0</v>
+      </c>
+      <c r="S86" s="2">
+        <v>1</v>
+      </c>
+      <c r="T86" s="2">
+        <v>0</v>
+      </c>
+      <c r="U86" s="2">
+        <v>2</v>
+      </c>
+      <c r="V86" s="2">
+        <v>0</v>
+      </c>
+      <c r="W86" s="2">
+        <v>3</v>
+      </c>
       <c r="X86" s="2"/>
       <c r="Y86" s="2"/>
       <c r="Z86" s="2"/>
@@ -8440,27 +8491,75 @@
       <c r="AF86" s="2"/>
     </row>
     <row r="87" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A87" s="2"/>
-      <c r="B87" s="2"/>
-      <c r="C87" s="2"/>
-      <c r="D87" s="2"/>
-      <c r="E87" s="2"/>
-      <c r="F87" s="2"/>
-      <c r="G87" s="2"/>
-      <c r="H87" s="2"/>
-      <c r="I87" s="2"/>
-      <c r="J87" s="2"/>
-      <c r="K87" s="2"/>
-      <c r="L87" s="2"/>
-      <c r="M87" s="2"/>
-      <c r="N87" s="2"/>
-      <c r="O87" s="2"/>
-      <c r="R87" s="2"/>
-      <c r="S87" s="2"/>
-      <c r="T87" s="2"/>
-      <c r="U87" s="2"/>
-      <c r="V87" s="2"/>
-      <c r="W87" s="2"/>
+      <c r="A87" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G87" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H87" s="6">
+        <v>15.4</v>
+      </c>
+      <c r="I87" s="6">
+        <v>2</v>
+      </c>
+      <c r="J87" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K87" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L87" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M87" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N87" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O87" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P87" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q87" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="R87" s="2">
+        <v>0</v>
+      </c>
+      <c r="S87" s="2">
+        <v>1</v>
+      </c>
+      <c r="T87" s="2">
+        <v>0</v>
+      </c>
+      <c r="U87" s="2">
+        <v>2</v>
+      </c>
+      <c r="V87" s="2">
+        <v>0</v>
+      </c>
+      <c r="W87" s="2">
+        <v>3</v>
+      </c>
       <c r="X87" s="2"/>
       <c r="Y87" s="2"/>
       <c r="Z87" s="2"/>
@@ -8472,27 +8571,75 @@
       <c r="AF87" s="2"/>
     </row>
     <row r="88" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A88" s="2"/>
-      <c r="B88" s="2"/>
-      <c r="C88" s="2"/>
-      <c r="D88" s="2"/>
-      <c r="E88" s="2"/>
-      <c r="F88" s="2"/>
-      <c r="G88" s="2"/>
-      <c r="H88" s="2"/>
-      <c r="I88" s="2"/>
-      <c r="J88" s="2"/>
-      <c r="K88" s="2"/>
-      <c r="L88" s="2"/>
-      <c r="M88" s="2"/>
-      <c r="N88" s="2"/>
-      <c r="O88" s="2"/>
-      <c r="R88" s="2"/>
-      <c r="S88" s="2"/>
-      <c r="T88" s="2"/>
-      <c r="U88" s="2"/>
-      <c r="V88" s="2"/>
-      <c r="W88" s="2"/>
+      <c r="A88" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G88" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H88" s="6">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="I88" s="6">
+        <v>4</v>
+      </c>
+      <c r="J88" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K88" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L88" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M88" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N88" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O88" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P88" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q88" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="R88" s="2">
+        <v>0</v>
+      </c>
+      <c r="S88" s="2">
+        <v>1</v>
+      </c>
+      <c r="T88" s="2">
+        <v>0</v>
+      </c>
+      <c r="U88" s="2">
+        <v>1</v>
+      </c>
+      <c r="V88" s="2">
+        <v>0</v>
+      </c>
+      <c r="W88" s="2">
+        <v>2</v>
+      </c>
       <c r="X88" s="2"/>
       <c r="Y88" s="2"/>
       <c r="Z88" s="2"/>
@@ -8504,27 +8651,75 @@
       <c r="AF88" s="2"/>
     </row>
     <row r="89" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A89" s="2"/>
-      <c r="B89" s="2"/>
-      <c r="C89" s="2"/>
-      <c r="D89" s="2"/>
-      <c r="E89" s="2"/>
-      <c r="F89" s="2"/>
-      <c r="G89" s="2"/>
-      <c r="H89" s="2"/>
-      <c r="I89" s="2"/>
-      <c r="J89" s="2"/>
-      <c r="K89" s="2"/>
-      <c r="L89" s="2"/>
-      <c r="M89" s="2"/>
-      <c r="N89" s="2"/>
-      <c r="O89" s="2"/>
-      <c r="R89" s="2"/>
-      <c r="S89" s="2"/>
-      <c r="T89" s="2"/>
-      <c r="U89" s="2"/>
-      <c r="V89" s="2"/>
-      <c r="W89" s="2"/>
+      <c r="A89" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F89" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G89" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H89" s="6">
+        <v>17.8</v>
+      </c>
+      <c r="I89" s="6">
+        <v>4</v>
+      </c>
+      <c r="J89" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K89" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L89" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M89" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N89" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O89" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P89" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q89" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="R89" s="2">
+        <v>0</v>
+      </c>
+      <c r="S89" s="2">
+        <v>1</v>
+      </c>
+      <c r="T89" s="2">
+        <v>0</v>
+      </c>
+      <c r="U89" s="2">
+        <v>2</v>
+      </c>
+      <c r="V89" s="2">
+        <v>0</v>
+      </c>
+      <c r="W89" s="2">
+        <v>2</v>
+      </c>
       <c r="X89" s="2"/>
       <c r="Y89" s="2"/>
       <c r="Z89" s="2"/>
@@ -8536,27 +8731,75 @@
       <c r="AF89" s="2"/>
     </row>
     <row r="90" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A90" s="2"/>
-      <c r="B90" s="2"/>
-      <c r="C90" s="2"/>
-      <c r="D90" s="2"/>
-      <c r="E90" s="2"/>
-      <c r="F90" s="2"/>
-      <c r="G90" s="2"/>
-      <c r="H90" s="2"/>
-      <c r="I90" s="2"/>
-      <c r="J90" s="2"/>
-      <c r="K90" s="2"/>
-      <c r="L90" s="2"/>
-      <c r="M90" s="2"/>
-      <c r="N90" s="2"/>
-      <c r="O90" s="2"/>
-      <c r="R90" s="2"/>
-      <c r="S90" s="2"/>
-      <c r="T90" s="2"/>
-      <c r="U90" s="2"/>
-      <c r="V90" s="2"/>
-      <c r="W90" s="2"/>
+      <c r="A90" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F90" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G90" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H90" s="6">
+        <v>20</v>
+      </c>
+      <c r="I90" s="6">
+        <v>2</v>
+      </c>
+      <c r="J90" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K90" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L90" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M90" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N90" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O90" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P90" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q90" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="R90" s="2">
+        <v>0</v>
+      </c>
+      <c r="S90" s="2">
+        <v>1</v>
+      </c>
+      <c r="T90" s="2">
+        <v>0</v>
+      </c>
+      <c r="U90" s="2">
+        <v>2</v>
+      </c>
+      <c r="V90" s="2">
+        <v>0</v>
+      </c>
+      <c r="W90" s="2">
+        <v>3</v>
+      </c>
       <c r="X90" s="2"/>
       <c r="Y90" s="2"/>
       <c r="Z90" s="2"/>
@@ -8568,59 +8811,146 @@
       <c r="AF90" s="2"/>
     </row>
     <row r="91" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A91" s="2"/>
-      <c r="B91" s="2"/>
-      <c r="C91" s="2"/>
-      <c r="D91" s="2"/>
-      <c r="E91" s="2"/>
-      <c r="F91" s="2"/>
-      <c r="G91" s="2"/>
-      <c r="H91" s="2"/>
-      <c r="I91" s="2"/>
-      <c r="J91" s="2"/>
-      <c r="K91" s="2"/>
-      <c r="L91" s="2"/>
-      <c r="M91" s="2"/>
-      <c r="N91" s="2"/>
-      <c r="O91" s="2"/>
-      <c r="R91" s="2"/>
-      <c r="S91" s="2"/>
-      <c r="T91" s="2"/>
-      <c r="U91" s="2"/>
-      <c r="V91" s="2"/>
-      <c r="W91" s="2"/>
-      <c r="X91" s="2"/>
-      <c r="Y91" s="2"/>
-      <c r="Z91" s="2"/>
-      <c r="AA91" s="2"/>
-      <c r="AB91" s="2"/>
-      <c r="AC91" s="2"/>
-      <c r="AD91" s="2"/>
-      <c r="AE91" s="2"/>
-      <c r="AF91" s="2"/>
+      <c r="A91" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E91" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F91" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G91" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H91" s="6">
+        <v>11.4</v>
+      </c>
+      <c r="I91" s="6">
+        <v>2</v>
+      </c>
+      <c r="J91" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K91" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L91" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M91" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N91" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O91" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P91" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q91" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="R91" s="2">
+        <v>0</v>
+      </c>
+      <c r="S91" s="2">
+        <v>1</v>
+      </c>
+      <c r="T91" s="2">
+        <v>0</v>
+      </c>
+      <c r="U91" s="2">
+        <v>1</v>
+      </c>
+      <c r="V91" s="2">
+        <v>0</v>
+      </c>
+      <c r="W91" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="92" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A92" s="2"/>
-      <c r="B92" s="2"/>
-      <c r="C92" s="2"/>
-      <c r="D92" s="2"/>
-      <c r="E92" s="2"/>
-      <c r="F92" s="2"/>
-      <c r="G92" s="2"/>
-      <c r="H92" s="2"/>
-      <c r="I92" s="2"/>
-      <c r="J92" s="2"/>
-      <c r="K92" s="2"/>
-      <c r="L92" s="2"/>
-      <c r="M92" s="2"/>
-      <c r="N92" s="2"/>
-      <c r="O92" s="2"/>
-      <c r="R92" s="2"/>
-      <c r="S92" s="2"/>
-      <c r="T92" s="2"/>
-      <c r="U92" s="2"/>
-      <c r="V92" s="2"/>
-      <c r="W92" s="2"/>
+      <c r="A92" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F92" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G92" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H92" s="2">
+        <v>11</v>
+      </c>
+      <c r="I92" s="2">
+        <v>-4</v>
+      </c>
+      <c r="J92" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K92" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L92" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M92" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N92" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O92" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P92" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q92" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="R92" s="2">
+        <v>0</v>
+      </c>
+      <c r="S92" s="2">
+        <v>1</v>
+      </c>
+      <c r="T92" s="2">
+        <v>0</v>
+      </c>
+      <c r="U92" s="2">
+        <v>1</v>
+      </c>
+      <c r="V92" s="2">
+        <v>0</v>
+      </c>
+      <c r="W92" s="2">
+        <v>2</v>
+      </c>
       <c r="X92" s="2"/>
       <c r="Y92" s="2"/>
       <c r="Z92" s="2"/>
@@ -8632,27 +8962,75 @@
       <c r="AF92" s="2"/>
     </row>
     <row r="93" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A93" s="2"/>
-      <c r="B93" s="2"/>
-      <c r="C93" s="2"/>
-      <c r="D93" s="2"/>
-      <c r="E93" s="2"/>
-      <c r="F93" s="2"/>
-      <c r="G93" s="2"/>
-      <c r="H93" s="2"/>
-      <c r="I93" s="2"/>
-      <c r="J93" s="2"/>
-      <c r="K93" s="2"/>
-      <c r="L93" s="2"/>
-      <c r="M93" s="2"/>
-      <c r="N93" s="2"/>
-      <c r="O93" s="2"/>
-      <c r="R93" s="2"/>
-      <c r="S93" s="2"/>
-      <c r="T93" s="2"/>
-      <c r="U93" s="2"/>
-      <c r="V93" s="2"/>
-      <c r="W93" s="2"/>
+      <c r="A93" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E93" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F93" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G93" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H93" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="I93" s="2">
+        <v>-6</v>
+      </c>
+      <c r="J93" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K93" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L93" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M93" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N93" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O93" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P93" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q93" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="R93" s="2">
+        <v>0</v>
+      </c>
+      <c r="S93" s="2">
+        <v>1</v>
+      </c>
+      <c r="T93" s="2">
+        <v>0</v>
+      </c>
+      <c r="U93" s="2">
+        <v>1</v>
+      </c>
+      <c r="V93" s="2">
+        <v>0</v>
+      </c>
+      <c r="W93" s="2">
+        <v>2</v>
+      </c>
       <c r="X93" s="2"/>
       <c r="Y93" s="2"/>
       <c r="Z93" s="2"/>
@@ -8664,27 +9042,75 @@
       <c r="AF93" s="2"/>
     </row>
     <row r="94" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A94" s="2"/>
-      <c r="B94" s="2"/>
-      <c r="C94" s="2"/>
-      <c r="D94" s="2"/>
-      <c r="E94" s="2"/>
-      <c r="F94" s="2"/>
-      <c r="G94" s="2"/>
-      <c r="H94" s="2"/>
-      <c r="I94" s="2"/>
-      <c r="J94" s="2"/>
-      <c r="K94" s="2"/>
-      <c r="L94" s="2"/>
-      <c r="M94" s="2"/>
-      <c r="N94" s="2"/>
-      <c r="O94" s="2"/>
-      <c r="R94" s="2"/>
-      <c r="S94" s="2"/>
-      <c r="T94" s="2"/>
-      <c r="U94" s="2"/>
-      <c r="V94" s="2"/>
-      <c r="W94" s="2"/>
+      <c r="A94" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G94" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H94" s="2">
+        <v>12.9</v>
+      </c>
+      <c r="I94" s="2">
+        <v>-6</v>
+      </c>
+      <c r="J94" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K94" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L94" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M94" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N94" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O94" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P94" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q94" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="R94" s="2">
+        <v>1</v>
+      </c>
+      <c r="S94" s="2">
+        <v>2</v>
+      </c>
+      <c r="T94" s="2">
+        <v>1</v>
+      </c>
+      <c r="U94" s="2">
+        <v>2</v>
+      </c>
+      <c r="V94" s="2">
+        <v>0</v>
+      </c>
+      <c r="W94" s="2">
+        <v>2</v>
+      </c>
       <c r="X94" s="2"/>
       <c r="Y94" s="2"/>
       <c r="Z94" s="2"/>
@@ -8696,27 +9122,75 @@
       <c r="AF94" s="2"/>
     </row>
     <row r="95" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A95" s="2"/>
-      <c r="B95" s="2"/>
-      <c r="C95" s="2"/>
-      <c r="D95" s="2"/>
-      <c r="E95" s="2"/>
-      <c r="F95" s="2"/>
-      <c r="G95" s="2"/>
-      <c r="H95" s="2"/>
-      <c r="I95" s="2"/>
-      <c r="J95" s="2"/>
-      <c r="K95" s="2"/>
-      <c r="L95" s="2"/>
-      <c r="M95" s="2"/>
-      <c r="N95" s="2"/>
-      <c r="O95" s="2"/>
-      <c r="R95" s="2"/>
-      <c r="S95" s="2"/>
-      <c r="T95" s="2"/>
-      <c r="U95" s="2"/>
-      <c r="V95" s="2"/>
-      <c r="W95" s="2"/>
+      <c r="A95" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G95" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H95" s="2">
+        <v>17.5</v>
+      </c>
+      <c r="I95" s="2">
+        <v>-6</v>
+      </c>
+      <c r="J95" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K95" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L95" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M95" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N95" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O95" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P95" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q95" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="R95" s="2">
+        <v>0</v>
+      </c>
+      <c r="S95" s="2">
+        <v>1</v>
+      </c>
+      <c r="T95" s="2">
+        <v>0</v>
+      </c>
+      <c r="U95" s="2">
+        <v>1</v>
+      </c>
+      <c r="V95" s="2">
+        <v>0</v>
+      </c>
+      <c r="W95" s="2">
+        <v>1</v>
+      </c>
       <c r="X95" s="2"/>
       <c r="Y95" s="2"/>
       <c r="Z95" s="2"/>
@@ -8728,27 +9202,75 @@
       <c r="AF95" s="2"/>
     </row>
     <row r="96" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A96" s="2"/>
-      <c r="B96" s="2"/>
-      <c r="C96" s="2"/>
-      <c r="D96" s="2"/>
-      <c r="E96" s="2"/>
-      <c r="F96" s="2"/>
-      <c r="G96" s="2"/>
-      <c r="H96" s="1"/>
-      <c r="I96" s="2"/>
-      <c r="J96" s="2"/>
-      <c r="K96" s="2"/>
-      <c r="L96" s="2"/>
-      <c r="M96" s="2"/>
-      <c r="N96" s="2"/>
-      <c r="O96" s="2"/>
-      <c r="R96" s="2"/>
-      <c r="S96" s="2"/>
-      <c r="T96" s="2"/>
-      <c r="U96" s="2"/>
-      <c r="V96" s="2"/>
-      <c r="W96" s="2"/>
+      <c r="A96" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G96" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H96" s="2">
+        <v>15</v>
+      </c>
+      <c r="I96" s="2">
+        <v>-6</v>
+      </c>
+      <c r="J96" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K96" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L96" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M96" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N96" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O96" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P96" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q96" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="R96" s="2">
+        <v>0</v>
+      </c>
+      <c r="S96" s="2">
+        <v>1</v>
+      </c>
+      <c r="T96" s="2">
+        <v>0</v>
+      </c>
+      <c r="U96" s="2">
+        <v>2</v>
+      </c>
+      <c r="V96" s="2">
+        <v>0</v>
+      </c>
+      <c r="W96" s="2">
+        <v>2</v>
+      </c>
       <c r="X96" s="2"/>
       <c r="Y96" s="2"/>
       <c r="Z96" s="2"/>
@@ -8760,27 +9282,75 @@
       <c r="AF96" s="2"/>
     </row>
     <row r="97" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A97" s="2"/>
-      <c r="B97" s="2"/>
-      <c r="C97" s="2"/>
-      <c r="D97" s="2"/>
-      <c r="E97" s="2"/>
-      <c r="F97" s="2"/>
-      <c r="G97" s="2"/>
-      <c r="H97" s="1"/>
-      <c r="I97" s="2"/>
-      <c r="J97" s="2"/>
-      <c r="K97" s="2"/>
-      <c r="L97" s="2"/>
-      <c r="M97" s="2"/>
-      <c r="N97" s="2"/>
-      <c r="O97" s="2"/>
-      <c r="R97" s="2"/>
-      <c r="S97" s="2"/>
-      <c r="T97" s="2"/>
-      <c r="U97" s="2"/>
-      <c r="V97" s="2"/>
-      <c r="W97" s="2"/>
+      <c r="A97" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E97" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F97" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G97" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H97" s="2">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="I97" s="2">
+        <v>-6</v>
+      </c>
+      <c r="J97" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K97" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L97" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M97" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N97" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O97" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P97" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q97" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="R97" s="2">
+        <v>1</v>
+      </c>
+      <c r="S97" s="2">
+        <v>1</v>
+      </c>
+      <c r="T97" s="2">
+        <v>1</v>
+      </c>
+      <c r="U97" s="2">
+        <v>2</v>
+      </c>
+      <c r="V97" s="2">
+        <v>0</v>
+      </c>
+      <c r="W97" s="2">
+        <v>2</v>
+      </c>
       <c r="X97" s="2"/>
       <c r="Y97" s="2"/>
       <c r="Z97" s="2"/>
@@ -8792,27 +9362,75 @@
       <c r="AF97" s="2"/>
     </row>
     <row r="98" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A98" s="2"/>
-      <c r="B98" s="2"/>
-      <c r="C98" s="2"/>
-      <c r="D98" s="2"/>
-      <c r="E98" s="2"/>
-      <c r="F98" s="2"/>
-      <c r="G98" s="2"/>
-      <c r="H98" s="1"/>
-      <c r="I98" s="2"/>
-      <c r="J98" s="2"/>
-      <c r="K98" s="2"/>
-      <c r="L98" s="2"/>
-      <c r="M98" s="2"/>
-      <c r="N98" s="2"/>
-      <c r="O98" s="2"/>
-      <c r="R98" s="2"/>
-      <c r="S98" s="2"/>
-      <c r="T98" s="2"/>
-      <c r="U98" s="2"/>
-      <c r="V98" s="2"/>
-      <c r="W98" s="2"/>
+      <c r="A98" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G98" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H98" s="2">
+        <v>12.2</v>
+      </c>
+      <c r="I98" s="2">
+        <v>-6</v>
+      </c>
+      <c r="J98" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K98" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L98" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M98" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N98" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O98" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P98" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q98" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="R98" s="2">
+        <v>0</v>
+      </c>
+      <c r="S98" s="2">
+        <v>1</v>
+      </c>
+      <c r="T98" s="2">
+        <v>0</v>
+      </c>
+      <c r="U98" s="2">
+        <v>1</v>
+      </c>
+      <c r="V98" s="2">
+        <v>0</v>
+      </c>
+      <c r="W98" s="2">
+        <v>1</v>
+      </c>
       <c r="X98" s="2"/>
       <c r="Y98" s="2"/>
       <c r="Z98" s="2"/>
@@ -8824,27 +9442,75 @@
       <c r="AF98" s="2"/>
     </row>
     <row r="99" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A99" s="2"/>
-      <c r="B99" s="2"/>
-      <c r="C99" s="2"/>
-      <c r="D99" s="2"/>
-      <c r="E99" s="2"/>
-      <c r="F99" s="2"/>
-      <c r="G99" s="2"/>
-      <c r="H99" s="1"/>
-      <c r="I99" s="2"/>
-      <c r="J99" s="2"/>
-      <c r="K99" s="2"/>
-      <c r="L99" s="2"/>
-      <c r="M99" s="2"/>
-      <c r="N99" s="2"/>
-      <c r="O99" s="2"/>
-      <c r="R99" s="2"/>
-      <c r="S99" s="2"/>
-      <c r="T99" s="2"/>
-      <c r="U99" s="2"/>
-      <c r="V99" s="2"/>
-      <c r="W99" s="2"/>
+      <c r="A99" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F99" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G99" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H99" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="I99" s="2">
+        <v>-6</v>
+      </c>
+      <c r="J99" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K99" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L99" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M99" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N99" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O99" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P99" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q99" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="R99" s="2">
+        <v>0</v>
+      </c>
+      <c r="S99" s="2">
+        <v>1</v>
+      </c>
+      <c r="T99" s="2">
+        <v>0</v>
+      </c>
+      <c r="U99" s="2">
+        <v>2</v>
+      </c>
+      <c r="V99" s="2">
+        <v>0</v>
+      </c>
+      <c r="W99" s="2">
+        <v>2</v>
+      </c>
       <c r="X99" s="2"/>
       <c r="Y99" s="2"/>
       <c r="Z99" s="2"/>
@@ -8856,27 +9522,75 @@
       <c r="AF99" s="2"/>
     </row>
     <row r="100" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A100" s="2"/>
-      <c r="B100" s="2"/>
-      <c r="C100" s="2"/>
-      <c r="D100" s="2"/>
-      <c r="E100" s="2"/>
-      <c r="F100" s="2"/>
-      <c r="G100" s="2"/>
-      <c r="H100" s="1"/>
-      <c r="I100" s="2"/>
-      <c r="J100" s="2"/>
-      <c r="K100" s="2"/>
-      <c r="L100" s="2"/>
-      <c r="M100" s="2"/>
-      <c r="N100" s="2"/>
-      <c r="O100" s="2"/>
-      <c r="R100" s="2"/>
-      <c r="S100" s="2"/>
-      <c r="T100" s="2"/>
-      <c r="U100" s="2"/>
-      <c r="V100" s="2"/>
-      <c r="W100" s="2"/>
+      <c r="A100" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G100" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H100" s="2">
+        <v>9.6</v>
+      </c>
+      <c r="I100" s="2">
+        <v>-6</v>
+      </c>
+      <c r="J100" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K100" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L100" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M100" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N100" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O100" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P100" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q100" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="R100" s="2">
+        <v>0</v>
+      </c>
+      <c r="S100" s="2">
+        <v>1</v>
+      </c>
+      <c r="T100" s="2">
+        <v>0</v>
+      </c>
+      <c r="U100" s="2">
+        <v>1</v>
+      </c>
+      <c r="V100" s="2">
+        <v>0</v>
+      </c>
+      <c r="W100" s="2">
+        <v>1</v>
+      </c>
       <c r="X100" s="2"/>
       <c r="Y100" s="2"/>
       <c r="Z100" s="2"/>
@@ -8888,27 +9602,75 @@
       <c r="AF100" s="2"/>
     </row>
     <row r="101" spans="1:32" x14ac:dyDescent="0.45">
-      <c r="A101" s="2"/>
-      <c r="B101" s="2"/>
-      <c r="C101" s="2"/>
-      <c r="D101" s="2"/>
-      <c r="E101" s="2"/>
-      <c r="F101" s="2"/>
-      <c r="G101" s="2"/>
-      <c r="H101" s="1"/>
-      <c r="I101" s="2"/>
-      <c r="J101" s="2"/>
-      <c r="K101" s="2"/>
-      <c r="L101" s="2"/>
-      <c r="M101" s="2"/>
-      <c r="N101" s="2"/>
-      <c r="O101" s="2"/>
-      <c r="R101" s="2"/>
-      <c r="S101" s="2"/>
-      <c r="T101" s="2"/>
-      <c r="U101" s="2"/>
-      <c r="V101" s="2"/>
-      <c r="W101" s="2"/>
+      <c r="A101" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F101" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G101" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H101" s="2">
+        <v>43.7</v>
+      </c>
+      <c r="I101" s="2">
+        <v>-6</v>
+      </c>
+      <c r="J101" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K101" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L101" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M101" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="N101" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O101" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="P101" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q101" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="R101" s="2">
+        <v>0</v>
+      </c>
+      <c r="S101" s="2">
+        <v>1</v>
+      </c>
+      <c r="T101" s="2">
+        <v>0</v>
+      </c>
+      <c r="U101" s="2">
+        <v>0</v>
+      </c>
+      <c r="V101" s="2">
+        <v>0</v>
+      </c>
+      <c r="W101" s="2">
+        <v>0</v>
+      </c>
       <c r="X101" s="2"/>
       <c r="Y101" s="2"/>
       <c r="Z101" s="2"/>

</xml_diff>